<commit_message>
Complete cutlet plots and data files for all 142 assemblies
All 142 assemblies now have cutlet plots (.png) and cutlet data files (.xlsx).
Master List.xlsx refreshed with links to all generated deliverables.
Building blocks completed: Source File (142/142), Cutlet Plot (142/142), Cutlet Data (142/142).

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Master/Master List.xlsx
+++ b/Master/Master List.xlsx
@@ -530,14 +530,14 @@
           <t>1941.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D4" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>1941r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>1941r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -567,14 +567,14 @@
           <t>2004.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D5" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>2004r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2004r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -604,14 +604,14 @@
           <t>2010.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D6" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>2010r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>2010r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -641,14 +641,14 @@
           <t>2028.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D7" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>2028r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>2028r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -678,14 +678,14 @@
           <t>2046.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>2046r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>2046r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -715,14 +715,14 @@
           <t>2053.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D9" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C9" s="4" t="inlineStr">
+        <is>
+          <t>2053r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>2053r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -752,14 +752,14 @@
           <t>2054.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D10" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>2054r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>2054r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -789,14 +789,14 @@
           <t>2070.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>2070r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>2070r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -826,14 +826,14 @@
           <t>2074.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D12" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>2074r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2074r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -863,14 +863,14 @@
           <t>2075.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D13" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>2075r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>2075r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -900,14 +900,14 @@
           <t>2077.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D14" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>2077r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2077r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -937,14 +937,14 @@
           <t>2079r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C15" s="4" t="inlineStr">
+        <is>
+          <t>2079r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="inlineStr">
+        <is>
+          <t>2079r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -974,14 +974,14 @@
           <t>2090.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D16" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C16" s="4" t="inlineStr">
+        <is>
+          <t>2090r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2090r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1011,14 +1011,14 @@
           <t>2091.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D17" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C17" s="4" t="inlineStr">
+        <is>
+          <t>2091r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D17" s="4" t="inlineStr">
+        <is>
+          <t>2091r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1048,14 +1048,14 @@
           <t>2095r02 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D18" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C18" s="4" t="inlineStr">
+        <is>
+          <t>2095r02_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>2095r02_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1085,14 +1085,14 @@
           <t>2095.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D19" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C19" s="4" t="inlineStr">
+        <is>
+          <t>2095r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D19" s="4" t="inlineStr">
+        <is>
+          <t>2095r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1122,14 +1122,14 @@
           <t>2096.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D20" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>2096r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2096r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1159,14 +1159,14 @@
           <t>2104.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t>2104r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t>2104r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1196,14 +1196,14 @@
           <t>2110.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D22" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C22" s="4" t="inlineStr">
+        <is>
+          <t>2110r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>2110r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1233,14 +1233,14 @@
           <t>2114r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C23" s="4" t="inlineStr">
+        <is>
+          <t>2114r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>2114r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1270,14 +1270,14 @@
           <t>2115.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D24" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C24" s="4" t="inlineStr">
+        <is>
+          <t>2115r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2115r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1307,14 +1307,14 @@
           <t>2117.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C25" s="4" t="inlineStr">
+        <is>
+          <t>2117r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>2117r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1344,14 +1344,14 @@
           <t>2119.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D26" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>2119r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>2119r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1381,14 +1381,14 @@
           <t>2120.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C27" s="4" t="inlineStr">
+        <is>
+          <t>2120r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>2120r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1418,14 +1418,14 @@
           <t>2121.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D28" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
+          <t>2121r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>2121r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1455,14 +1455,14 @@
           <t>2122.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>2122r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>2122r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1492,14 +1492,14 @@
           <t>2124.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
+          <t>2124r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>2124r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1529,14 +1529,14 @@
           <t>2126r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
+          <t>2126r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D31" s="4" t="inlineStr">
+        <is>
+          <t>2126r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1566,14 +1566,14 @@
           <t>2131.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D32" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C32" s="4" t="inlineStr">
+        <is>
+          <t>2131r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>2131r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1603,14 +1603,14 @@
           <t>2137r2 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C33" s="4" t="inlineStr">
+        <is>
+          <t>2137r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D33" s="4" t="inlineStr">
+        <is>
+          <t>2137r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1640,14 +1640,14 @@
           <t>2140.r3 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C34" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C34" s="4" t="inlineStr">
+        <is>
+          <t>2140r3_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>2140r3_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1677,14 +1677,14 @@
           <t>2140.r4 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C35" s="4" t="inlineStr">
+        <is>
+          <t>2140r4_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D35" s="4" t="inlineStr">
+        <is>
+          <t>2140r4_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1714,14 +1714,14 @@
           <t>2141.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D36" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C36" s="4" t="inlineStr">
+        <is>
+          <t>2141r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>2141r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1751,14 +1751,14 @@
           <t>2142.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C37" s="4" t="inlineStr">
+        <is>
+          <t>2142r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D37" s="4" t="inlineStr">
+        <is>
+          <t>2142r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1788,14 +1788,14 @@
           <t>2143.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C38" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D38" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C38" s="4" t="inlineStr">
+        <is>
+          <t>2143r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>2143r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -1825,14 +1825,14 @@
           <t>2145.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C39" s="4" t="inlineStr">
+        <is>
+          <t>2145r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D39" s="4" t="inlineStr">
+        <is>
+          <t>2145r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -1862,14 +1862,14 @@
           <t>2148.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D40" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C40" s="4" t="inlineStr">
+        <is>
+          <t>2148r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>2148r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -1899,14 +1899,14 @@
           <t>2152.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C41" s="4" t="inlineStr">
+        <is>
+          <t>2152r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D41" s="4" t="inlineStr">
+        <is>
+          <t>2152r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -1936,14 +1936,14 @@
           <t>2153.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C42" s="4" t="inlineStr">
+        <is>
+          <t>2153r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>2153r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -1973,14 +1973,14 @@
           <t>2154.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C43" s="4" t="inlineStr">
+        <is>
+          <t>2154r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D43" s="4" t="inlineStr">
+        <is>
+          <t>2154r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2010,14 +2010,14 @@
           <t>2157.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C44" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D44" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C44" s="4" t="inlineStr">
+        <is>
+          <t>2157r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>2157r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2047,14 +2047,14 @@
           <t>2158.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C45" s="4" t="inlineStr">
+        <is>
+          <t>2158r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D45" s="4" t="inlineStr">
+        <is>
+          <t>2158r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2084,14 +2084,14 @@
           <t>2160.r5 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D46" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C46" s="4" t="inlineStr">
+        <is>
+          <t>2160r5_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>2160r5_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2121,14 +2121,14 @@
           <t>2164.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C47" s="4" t="inlineStr">
+        <is>
+          <t>2164r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D47" s="4" t="inlineStr">
+        <is>
+          <t>2164r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2158,14 +2158,14 @@
           <t>2169.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D48" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C48" s="4" t="inlineStr">
+        <is>
+          <t>2169r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>2169r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2195,14 +2195,14 @@
           <t>2172r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C49" s="4" t="inlineStr">
+        <is>
+          <t>2172r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D49" s="4" t="inlineStr">
+        <is>
+          <t>2172r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2232,14 +2232,14 @@
           <t>2173.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D50" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>2173r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>2173r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2269,14 +2269,14 @@
           <t>2174.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>2174r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D51" s="4" t="inlineStr">
+        <is>
+          <t>2174r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2311,9 +2311,9 @@
           <t>2176r06_cutlet_plot.png</t>
         </is>
       </c>
-      <c r="D52" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>2176r06_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -2343,14 +2343,14 @@
           <t>2177.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>2177r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D53" s="4" t="inlineStr">
+        <is>
+          <t>2177r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2380,14 +2380,14 @@
           <t>2179.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C54" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D54" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C54" s="4" t="inlineStr">
+        <is>
+          <t>2179r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>2179r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2417,14 +2417,14 @@
           <t>2180.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C55" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D55" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C55" s="4" t="inlineStr">
+        <is>
+          <t>2180r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D55" s="4" t="inlineStr">
+        <is>
+          <t>2180r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2454,14 +2454,14 @@
           <t>2181.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C56" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D56" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C56" s="4" t="inlineStr">
+        <is>
+          <t>2181r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>2181r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2491,14 +2491,14 @@
           <t>2184r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C57" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D57" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C57" s="4" t="inlineStr">
+        <is>
+          <t>2184r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D57" s="4" t="inlineStr">
+        <is>
+          <t>2184r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2528,14 +2528,14 @@
           <t>2185.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C58" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D58" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>2185r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>2185r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2565,14 +2565,14 @@
           <t>2186.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C59" s="4" t="inlineStr">
+        <is>
+          <t>2186r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D59" s="4" t="inlineStr">
+        <is>
+          <t>2186r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2602,14 +2602,14 @@
           <t>2188.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C60" s="4" t="inlineStr">
+        <is>
+          <t>2188r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>2188r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2639,14 +2639,14 @@
           <t>2190.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C61" s="4" t="inlineStr">
+        <is>
+          <t>2190r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D61" s="4" t="inlineStr">
+        <is>
+          <t>2190r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2676,14 +2676,14 @@
           <t>2192r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C62" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D62" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C62" s="4" t="inlineStr">
+        <is>
+          <t>2192r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>2192r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2713,14 +2713,14 @@
           <t>2193.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C63" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D63" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C63" s="4" t="inlineStr">
+        <is>
+          <t>2193r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D63" s="4" t="inlineStr">
+        <is>
+          <t>2193r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2750,14 +2750,14 @@
           <t>2194.r3 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C64" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D64" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>2194r3_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>2194r3_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2787,14 +2787,14 @@
           <t>2195.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C65" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D65" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C65" s="4" t="inlineStr">
+        <is>
+          <t>2195r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D65" s="4" t="inlineStr">
+        <is>
+          <t>2195r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2824,14 +2824,14 @@
           <t>2196.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C66" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D66" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C66" s="4" t="inlineStr">
+        <is>
+          <t>2196r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>2196r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2861,14 +2861,14 @@
           <t>2198.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C67" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D67" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C67" s="4" t="inlineStr">
+        <is>
+          <t>2198r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D67" s="4" t="inlineStr">
+        <is>
+          <t>2198r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2898,14 +2898,14 @@
           <t>2205.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C68" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D68" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C68" s="4" t="inlineStr">
+        <is>
+          <t>2205r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>2205r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2935,14 +2935,14 @@
           <t>2206.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C69" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D69" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C69" s="4" t="inlineStr">
+        <is>
+          <t>2206r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D69" s="4" t="inlineStr">
+        <is>
+          <t>2206r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2972,14 +2972,14 @@
           <t>2207.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C70" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D70" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C70" s="4" t="inlineStr">
+        <is>
+          <t>2207r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>2207r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -3009,14 +3009,14 @@
           <t>2208.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C71" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D71" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C71" s="4" t="inlineStr">
+        <is>
+          <t>2208r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D71" s="4" t="inlineStr">
+        <is>
+          <t>2208r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3046,14 +3046,14 @@
           <t>2209.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D72" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C72" s="4" t="inlineStr">
+        <is>
+          <t>2209r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>2209r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3083,14 +3083,14 @@
           <t>2210.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C73" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D73" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C73" s="4" t="inlineStr">
+        <is>
+          <t>2210r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D73" s="4" t="inlineStr">
+        <is>
+          <t>2210r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3120,14 +3120,14 @@
           <t>2216.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C74" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D74" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C74" s="4" t="inlineStr">
+        <is>
+          <t>2216r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>2216r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3157,14 +3157,14 @@
           <t>2217.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C75" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D75" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C75" s="4" t="inlineStr">
+        <is>
+          <t>2217r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D75" s="4" t="inlineStr">
+        <is>
+          <t>2217r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3194,14 +3194,14 @@
           <t>2218.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D76" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C76" s="4" t="inlineStr">
+        <is>
+          <t>2218r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>2218r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3231,14 +3231,14 @@
           <t>2220.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D77" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C77" s="4" t="inlineStr">
+        <is>
+          <t>2220r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D77" s="4" t="inlineStr">
+        <is>
+          <t>2220r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3268,14 +3268,14 @@
           <t>2224.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D78" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C78" s="4" t="inlineStr">
+        <is>
+          <t>2224r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>2224r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3305,14 +3305,14 @@
           <t>2225.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D79" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C79" s="4" t="inlineStr">
+        <is>
+          <t>2225r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D79" s="4" t="inlineStr">
+        <is>
+          <t>2225r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3342,14 +3342,14 @@
           <t>2226r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D80" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C80" s="4" t="inlineStr">
+        <is>
+          <t>2226r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>2226r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3379,14 +3379,14 @@
           <t>2227.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C81" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D81" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C81" s="4" t="inlineStr">
+        <is>
+          <t>2227r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D81" s="4" t="inlineStr">
+        <is>
+          <t>2227r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3416,14 +3416,14 @@
           <t>2231.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D82" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C82" s="4" t="inlineStr">
+        <is>
+          <t>2231r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>2231r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3453,14 +3453,14 @@
           <t>2232.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C83" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D83" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C83" s="4" t="inlineStr">
+        <is>
+          <t>2232r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D83" s="4" t="inlineStr">
+        <is>
+          <t>2232r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3490,14 +3490,14 @@
           <t>2234r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C84" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D84" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C84" s="4" t="inlineStr">
+        <is>
+          <t>2234r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>2234r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3527,14 +3527,14 @@
           <t>2235.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C85" s="4" t="inlineStr">
+        <is>
+          <t>2235r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D85" s="4" t="inlineStr">
+        <is>
+          <t>2235r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -3564,14 +3564,14 @@
           <t>2236.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D86" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C86" s="4" t="inlineStr">
+        <is>
+          <t>2236r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>2236r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3601,14 +3601,14 @@
           <t>2240r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C87" s="4" t="inlineStr">
+        <is>
+          <t>2240r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D87" s="4" t="inlineStr">
+        <is>
+          <t>2240r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3638,14 +3638,14 @@
           <t>2241.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C88" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D88" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>2241r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>2241r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -3675,14 +3675,14 @@
           <t>2242r0 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C89" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D89" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>2242r0_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D89" s="4" t="inlineStr">
+        <is>
+          <t>2242r0_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -3712,14 +3712,14 @@
           <t>2247.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D90" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>2247r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>2247r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -3749,14 +3749,14 @@
           <t>2249r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C91" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D91" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C91" s="4" t="inlineStr">
+        <is>
+          <t>2249r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D91" s="4" t="inlineStr">
+        <is>
+          <t>2249r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -3786,14 +3786,14 @@
           <t>2251.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C92" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D92" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C92" s="4" t="inlineStr">
+        <is>
+          <t>2251r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>2251r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -3823,14 +3823,14 @@
           <t>2252r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C93" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D93" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C93" s="4" t="inlineStr">
+        <is>
+          <t>2252r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D93" s="4" t="inlineStr">
+        <is>
+          <t>2252r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -3860,14 +3860,14 @@
           <t>2256.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D94" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C94" s="4" t="inlineStr">
+        <is>
+          <t>2256r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>2256r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -3897,14 +3897,14 @@
           <t>2265r0 w Rippers Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C95" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D95" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C95" s="4" t="inlineStr">
+        <is>
+          <t>2265r0 w Rippers_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D95" s="4" t="inlineStr">
+        <is>
+          <t>2265r0 w Rippers_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -3934,14 +3934,14 @@
           <t>2265.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C96" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D96" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C96" s="4" t="inlineStr">
+        <is>
+          <t>2265r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>2265r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -3971,14 +3971,14 @@
           <t>2266.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C97" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D97" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C97" s="4" t="inlineStr">
+        <is>
+          <t>2266r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D97" s="4" t="inlineStr">
+        <is>
+          <t>2266r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -4008,14 +4008,14 @@
           <t>2267.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C98" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D98" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C98" s="4" t="inlineStr">
+        <is>
+          <t>2267r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>2267r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -4045,14 +4045,14 @@
           <t>2268.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C99" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D99" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>2268r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D99" s="4" t="inlineStr">
+        <is>
+          <t>2268r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -4082,14 +4082,14 @@
           <t>2268.r3 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D100" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>2268r3_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>2268r3_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -4119,14 +4119,14 @@
           <t>2270.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C101" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D101" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>2270r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D101" s="4" t="inlineStr">
+        <is>
+          <t>2270r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -4156,14 +4156,14 @@
           <t>2272.r2 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C102" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D102" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C102" s="4" t="inlineStr">
+        <is>
+          <t>2272r2_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>2272r2_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -4193,14 +4193,14 @@
           <t>2362r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D103" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C103" s="4" t="inlineStr">
+        <is>
+          <t>2362r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D103" s="4" t="inlineStr">
+        <is>
+          <t>2362r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -4230,14 +4230,14 @@
           <t>2381r01 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C104" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D104" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C104" s="4" t="inlineStr">
+        <is>
+          <t>2381r01_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>2381r01_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -4267,14 +4267,14 @@
           <t>2381.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C105" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D105" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C105" s="4" t="inlineStr">
+        <is>
+          <t>2381r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D105" s="4" t="inlineStr">
+        <is>
+          <t>2381r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -4304,14 +4304,14 @@
           <t>2556r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C106" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D106" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C106" s="4" t="inlineStr">
+        <is>
+          <t>2556r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>2556r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -4341,14 +4341,14 @@
           <t>2556r00 XH23F Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C107" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D107" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C107" s="4" t="inlineStr">
+        <is>
+          <t>2556r00 XH23F_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D107" s="4" t="inlineStr">
+        <is>
+          <t>2556r00 XH23F_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -4378,14 +4378,14 @@
           <t>2746r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C108" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D108" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C108" s="4" t="inlineStr">
+        <is>
+          <t>2746r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>2746r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -4415,14 +4415,14 @@
           <t>3219r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C109" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D109" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C109" s="4" t="inlineStr">
+        <is>
+          <t>3219r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D109" s="4" t="inlineStr">
+        <is>
+          <t>3219r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -4452,14 +4452,14 @@
           <t>3336r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C110" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D110" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>3336r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>3336r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
@@ -4489,14 +4489,14 @@
           <t>3336r00c3 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C111" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D111" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>3336r00c3_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D111" s="4" t="inlineStr">
+        <is>
+          <t>3336r00c3_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
@@ -4526,14 +4526,14 @@
           <t>3449r00 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C112" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D112" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>3449r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>3449r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
@@ -4563,14 +4563,14 @@
           <t>3943.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C113" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D113" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C113" s="4" t="inlineStr">
+        <is>
+          <t>3943r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D113" s="4" t="inlineStr">
+        <is>
+          <t>3943r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
@@ -4600,14 +4600,14 @@
           <t>4149r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C114" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D114" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C114" s="4" t="inlineStr">
+        <is>
+          <t>4149r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>4149r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
@@ -4637,14 +4637,14 @@
           <t>4206.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D115" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C115" s="4" t="inlineStr">
+        <is>
+          <t>4206r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D115" s="4" t="inlineStr">
+        <is>
+          <t>4206r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -4674,14 +4674,14 @@
           <t>4288r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C116" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D116" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C116" s="4" t="inlineStr">
+        <is>
+          <t>4288r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>4288r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
@@ -4711,14 +4711,14 @@
           <t>4538r0 Min Engagement v6.10.xlsm</t>
         </is>
       </c>
-      <c r="C117" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D117" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C117" s="4" t="inlineStr">
+        <is>
+          <t>4538r0_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D117" s="4" t="inlineStr">
+        <is>
+          <t>4538r0_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
@@ -4748,14 +4748,14 @@
           <t>4538r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C118" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D118" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C118" s="4" t="inlineStr">
+        <is>
+          <t>4538r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>4538r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
@@ -4785,14 +4785,14 @@
           <t>4720r01 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C119" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D119" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C119" s="4" t="inlineStr">
+        <is>
+          <t>4720r01_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D119" s="4" t="inlineStr">
+        <is>
+          <t>4720r01_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
@@ -4822,14 +4822,14 @@
           <t>4720r1 Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C120" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D120" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C120" s="4" t="inlineStr">
+        <is>
+          <t>4720r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>4720r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
@@ -4859,14 +4859,14 @@
           <t>4796r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C121" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D121" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>4796r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D121" s="4" t="inlineStr">
+        <is>
+          <t>4796r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
@@ -4896,14 +4896,14 @@
           <t>5131r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C122" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D122" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>5131r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>5131r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
@@ -4933,14 +4933,14 @@
           <t>5132r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C123" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D123" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>5132r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D123" s="4" t="inlineStr">
+        <is>
+          <t>5132r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
@@ -4970,14 +4970,14 @@
           <t>5481r0 Rev Min Engagement v6.08.xlsm</t>
         </is>
       </c>
-      <c r="C124" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D124" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C124" s="4" t="inlineStr">
+        <is>
+          <t>5481r0 Rev_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>5481r0 Rev_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
@@ -5007,14 +5007,14 @@
           <t>5646r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C125" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D125" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C125" s="4" t="inlineStr">
+        <is>
+          <t>5646r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D125" s="4" t="inlineStr">
+        <is>
+          <t>5646r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
@@ -5044,14 +5044,14 @@
           <t>5674r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C126" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D126" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C126" s="4" t="inlineStr">
+        <is>
+          <t>5674r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>5674r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
@@ -5081,14 +5081,14 @@
           <t>5749r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C127" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D127" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C127" s="4" t="inlineStr">
+        <is>
+          <t>5749r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D127" s="4" t="inlineStr">
+        <is>
+          <t>5749r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
@@ -5118,14 +5118,14 @@
           <t>5911r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C128" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D128" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C128" s="4" t="inlineStr">
+        <is>
+          <t>5911r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>5911r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
@@ -5155,14 +5155,14 @@
           <t>6135r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C129" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D129" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C129" s="4" t="inlineStr">
+        <is>
+          <t>6135r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D129" s="4" t="inlineStr">
+        <is>
+          <t>6135r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
@@ -5192,14 +5192,14 @@
           <t>6150r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C130" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D130" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C130" s="4" t="inlineStr">
+        <is>
+          <t>6150r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>6150r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
@@ -5229,14 +5229,14 @@
           <t>6150r01 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C131" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D131" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C131" s="4" t="inlineStr">
+        <is>
+          <t>6150r01_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D131" s="4" t="inlineStr">
+        <is>
+          <t>6150r01_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
@@ -5266,14 +5266,14 @@
           <t>6207.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C132" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D132" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C132" s="4" t="inlineStr">
+        <is>
+          <t>6207r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>6207r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
@@ -5303,14 +5303,14 @@
           <t>6513r0 Min Engagement v6.10.xlsm</t>
         </is>
       </c>
-      <c r="C133" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D133" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C133" s="4" t="inlineStr">
+        <is>
+          <t>6513r0_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D133" s="4" t="inlineStr">
+        <is>
+          <t>6513r0_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
@@ -5340,14 +5340,14 @@
           <t>6513r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C134" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D134" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C134" s="4" t="inlineStr">
+        <is>
+          <t>6513r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>6513r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
@@ -5377,14 +5377,14 @@
           <t>6653r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C135" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D135" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C135" s="4" t="inlineStr">
+        <is>
+          <t>6653r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D135" s="4" t="inlineStr">
+        <is>
+          <t>6653r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
@@ -5414,14 +5414,14 @@
           <t>6841r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C136" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D136" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C136" s="4" t="inlineStr">
+        <is>
+          <t>6841r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>6841r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E136" s="5" t="inlineStr">
@@ -5451,14 +5451,14 @@
           <t>7182r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C137" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D137" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C137" s="4" t="inlineStr">
+        <is>
+          <t>7182r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D137" s="4" t="inlineStr">
+        <is>
+          <t>7182r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
@@ -5488,14 +5488,14 @@
           <t>7273r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C138" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D138" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>7273r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>7273r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
@@ -5525,14 +5525,14 @@
           <t>7823r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C139" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D139" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>7823r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D139" s="4" t="inlineStr">
+        <is>
+          <t>7823r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
@@ -5562,14 +5562,14 @@
           <t>8479.r1 Min Engagement v6.07.xlsm</t>
         </is>
       </c>
-      <c r="C140" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D140" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>8479r1_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>8479r1_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E140" s="5" t="inlineStr">
@@ -5599,14 +5599,14 @@
           <t>8896r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C141" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D141" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C141" s="4" t="inlineStr">
+        <is>
+          <t>8896r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D141" s="4" t="inlineStr">
+        <is>
+          <t>8896r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
@@ -5636,14 +5636,14 @@
           <t>9023r00 Min Engagement v7.01.xlsm</t>
         </is>
       </c>
-      <c r="C142" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D142" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C142" s="4" t="inlineStr">
+        <is>
+          <t>9023r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>9023r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
@@ -5673,14 +5673,14 @@
           <t>9387r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C143" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D143" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C143" s="4" t="inlineStr">
+        <is>
+          <t>9387r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D143" s="4" t="inlineStr">
+        <is>
+          <t>9387r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
@@ -5710,14 +5710,14 @@
           <t>9692r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C144" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D144" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C144" s="4" t="inlineStr">
+        <is>
+          <t>9692r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>9692r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
@@ -5747,14 +5747,14 @@
           <t>9944r00 Min Engagement v8.01.xlsm</t>
         </is>
       </c>
-      <c r="C145" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="D145" s="5" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C145" s="4" t="inlineStr">
+        <is>
+          <t>9944r00_cutlet_plot.png</t>
+        </is>
+      </c>
+      <c r="D145" s="4" t="inlineStr">
+        <is>
+          <t>9944r00_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">
@@ -5779,148 +5779,431 @@
   </mergeCells>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B121" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B122" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B123" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C4" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C5" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D5" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C6" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D6" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C7" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D7" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C8" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D8" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C9" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D9" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C10" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D10" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C11" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D11" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B12" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C12" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D12" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B13" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C13" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D13" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B14" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C14" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D14" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B15" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C15" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D15" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D16" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C18" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D18" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D19" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D21" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C26" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D29" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C31" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D31" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B33" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C33" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B34" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D34" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D37" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D39" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B42" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B43" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B44" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B45" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B46" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C46" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B47" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C47" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B48" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C48" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B49" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C49" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B50" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C50" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D50" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B51" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C51" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D51" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B52" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C52" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D52" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B53" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C53" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D53" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B54" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C54" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B55" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C55" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B56" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C56" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B57" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C57" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B58" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C58" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B59" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C59" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B60" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C60" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B61" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C61" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B62" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C62" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B63" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C63" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B64" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C64" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B65" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C65" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B66" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B67" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C67" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B68" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C68" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B69" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B70" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B71" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B72" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B73" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C73" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B74" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C74" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B75" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C75" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B76" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C76" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B77" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C77" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B78" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B79" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C79" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B80" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C80" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B81" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C81" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B82" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C82" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B83" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C83" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B84" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C84" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B85" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C85" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B86" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C86" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B87" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C87" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B88" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C88" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B89" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C89" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B90" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C90" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B91" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C91" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B92" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C92" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B93" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C93" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B94" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C94" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B95" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C95" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B96" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C96" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B97" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C97" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B98" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C98" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B99" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C99" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B100" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C100" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B101" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C101" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B102" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C102" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B103" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C103" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B104" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C104" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B105" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C105" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B106" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C106" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B107" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C107" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B108" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C108" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B109" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C109" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B110" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C110" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B111" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C111" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B112" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C112" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B113" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C113" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B114" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C114" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B115" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C115" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B116" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C116" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B117" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C117" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B118" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C118" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B119" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C119" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B120" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C120" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B121" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C121" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B122" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C122" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B123" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C123" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B124" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C124" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B125" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C125" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B126" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C126" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B127" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C127" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B128" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C128" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B129" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C129" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B130" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C130" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B131" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C131" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B132" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C132" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B133" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C133" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B134" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C134" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B135" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C135" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B136" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C136" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B137" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C137" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B138" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C138" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B139" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C139" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B140" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C140" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B141" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C141" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B142" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C142" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B143" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C143" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B144" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C144" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B145" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="C145" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId426"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Exclude back-reamers/wear pads, rename files to include IPR
- Added Z-gap detection (>1 inch) to exclude non-drilling cutters
  (back-reamers, wear pad elements) from all cutlet computations
- Renamed output files to "<assy> @ <IPR> IPR_cutlet_plot.png" format
- Regenerated all 142 cutlet plots and data files
- Refreshed Master List.xlsx with updated file links

https://claude.ai/code/session_01N8TFjZHRi9fPjGEUiAzPPF
</commit_message>
<xml_diff>
--- a/Master/Master List.xlsx
+++ b/Master/Master List.xlsx
@@ -532,12 +532,12 @@
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>1941r2_cutlet_plot.png</t>
+          <t>1941r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>1941r2_cutlet_data.xlsx</t>
+          <t>1941r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -569,12 +569,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>2004r1_cutlet_plot.png</t>
+          <t>2004r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>2004r1_cutlet_data.xlsx</t>
+          <t>2004r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr">
@@ -606,12 +606,12 @@
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>2010r2_cutlet_plot.png</t>
+          <t>2010r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2010r2_cutlet_data.xlsx</t>
+          <t>2010r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr">
@@ -643,12 +643,12 @@
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>2028r1_cutlet_plot.png</t>
+          <t>2028r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>2028r1_cutlet_data.xlsx</t>
+          <t>2028r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -680,12 +680,12 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>2046r1_cutlet_plot.png</t>
+          <t>2046r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2046r1_cutlet_data.xlsx</t>
+          <t>2046r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -717,12 +717,12 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>2053r1_cutlet_plot.png</t>
+          <t>2053r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>2053r1_cutlet_data.xlsx</t>
+          <t>2053r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -754,12 +754,12 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>2054r1_cutlet_plot.png</t>
+          <t>2054r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2054r1_cutlet_data.xlsx</t>
+          <t>2054r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E10" s="5" t="inlineStr">
@@ -791,12 +791,12 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>2070r1_cutlet_plot.png</t>
+          <t>2070r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>2070r1_cutlet_data.xlsx</t>
+          <t>2070r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -828,12 +828,12 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>2074r1_cutlet_plot.png</t>
+          <t>2074r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2074r1_cutlet_data.xlsx</t>
+          <t>2074r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -865,12 +865,12 @@
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>2075r1_cutlet_plot.png</t>
+          <t>2075r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>2075r1_cutlet_data.xlsx</t>
+          <t>2075r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr">
@@ -902,12 +902,12 @@
       </c>
       <c r="C14" s="4" t="inlineStr">
         <is>
-          <t>2077r1_cutlet_plot.png</t>
+          <t>2077r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2077r1_cutlet_data.xlsx</t>
+          <t>2077r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E14" s="5" t="inlineStr">
@@ -939,12 +939,12 @@
       </c>
       <c r="C15" s="4" t="inlineStr">
         <is>
-          <t>2079r1_cutlet_plot.png</t>
+          <t>2079r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D15" s="4" t="inlineStr">
         <is>
-          <t>2079r1_cutlet_data.xlsx</t>
+          <t>2079r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E15" s="5" t="inlineStr">
@@ -976,12 +976,12 @@
       </c>
       <c r="C16" s="4" t="inlineStr">
         <is>
-          <t>2090r1_cutlet_plot.png</t>
+          <t>2090r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2090r1_cutlet_data.xlsx</t>
+          <t>2090r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E16" s="5" t="inlineStr">
@@ -1013,12 +1013,12 @@
       </c>
       <c r="C17" s="4" t="inlineStr">
         <is>
-          <t>2091r1_cutlet_plot.png</t>
+          <t>2091r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>2091r1_cutlet_data.xlsx</t>
+          <t>2091r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E17" s="5" t="inlineStr">
@@ -1050,12 +1050,12 @@
       </c>
       <c r="C18" s="4" t="inlineStr">
         <is>
-          <t>2095r02_cutlet_plot.png</t>
+          <t>2095r02 @ 0.190 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2095r02_cutlet_data.xlsx</t>
+          <t>2095r02 @ 0.190 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E18" s="5" t="inlineStr">
@@ -1087,12 +1087,12 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>2095r1_cutlet_plot.png</t>
+          <t>2095r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>2095r1_cutlet_data.xlsx</t>
+          <t>2095r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E19" s="5" t="inlineStr">
@@ -1124,12 +1124,12 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>2096r1_cutlet_plot.png</t>
+          <t>2096r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2096r1_cutlet_data.xlsx</t>
+          <t>2096r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">
@@ -1161,12 +1161,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>2104r1_cutlet_plot.png</t>
+          <t>2104r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>2104r1_cutlet_data.xlsx</t>
+          <t>2104r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E21" s="5" t="inlineStr">
@@ -1198,12 +1198,12 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>2110r1_cutlet_plot.png</t>
+          <t>2110r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2110r1_cutlet_data.xlsx</t>
+          <t>2110r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>2114r1_cutlet_plot.png</t>
+          <t>2114r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>2114r1_cutlet_data.xlsx</t>
+          <t>2114r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E23" s="5" t="inlineStr">
@@ -1272,12 +1272,12 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>2115r1_cutlet_plot.png</t>
+          <t>2115r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2115r1_cutlet_data.xlsx</t>
+          <t>2115r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E24" s="5" t="inlineStr">
@@ -1309,12 +1309,12 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>2117r1_cutlet_plot.png</t>
+          <t>2117r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>2117r1_cutlet_data.xlsx</t>
+          <t>2117r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E25" s="5" t="inlineStr">
@@ -1346,12 +1346,12 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>2119r1_cutlet_plot.png</t>
+          <t>2119r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2119r1_cutlet_data.xlsx</t>
+          <t>2119r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -1383,12 +1383,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>2120r1_cutlet_plot.png</t>
+          <t>2120r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>2120r1_cutlet_data.xlsx</t>
+          <t>2120r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -1420,12 +1420,12 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>2121r1_cutlet_plot.png</t>
+          <t>2121r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2121r1_cutlet_data.xlsx</t>
+          <t>2121r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -1457,12 +1457,12 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>2122r1_cutlet_plot.png</t>
+          <t>2122r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>2122r1_cutlet_data.xlsx</t>
+          <t>2122r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E29" s="5" t="inlineStr">
@@ -1494,12 +1494,12 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
-          <t>2124r2_cutlet_plot.png</t>
+          <t>2124r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2124r2_cutlet_data.xlsx</t>
+          <t>2124r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E30" s="5" t="inlineStr">
@@ -1531,12 +1531,12 @@
       </c>
       <c r="C31" s="4" t="inlineStr">
         <is>
-          <t>2126r1_cutlet_plot.png</t>
+          <t>2126r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D31" s="4" t="inlineStr">
         <is>
-          <t>2126r1_cutlet_data.xlsx</t>
+          <t>2126r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E31" s="5" t="inlineStr">
@@ -1568,12 +1568,12 @@
       </c>
       <c r="C32" s="4" t="inlineStr">
         <is>
-          <t>2131r1_cutlet_plot.png</t>
+          <t>2131r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2131r1_cutlet_data.xlsx</t>
+          <t>2131r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E32" s="5" t="inlineStr">
@@ -1605,12 +1605,12 @@
       </c>
       <c r="C33" s="4" t="inlineStr">
         <is>
-          <t>2137r2_cutlet_plot.png</t>
+          <t>2137r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D33" s="4" t="inlineStr">
         <is>
-          <t>2137r2_cutlet_data.xlsx</t>
+          <t>2137r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -1642,12 +1642,12 @@
       </c>
       <c r="C34" s="4" t="inlineStr">
         <is>
-          <t>2140r3_cutlet_plot.png</t>
+          <t>2140r3 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>2140r3_cutlet_data.xlsx</t>
+          <t>2140r3 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E34" s="5" t="inlineStr">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="C35" s="4" t="inlineStr">
         <is>
-          <t>2140r4_cutlet_plot.png</t>
+          <t>2140r4 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D35" s="4" t="inlineStr">
         <is>
-          <t>2140r4_cutlet_data.xlsx</t>
+          <t>2140r4 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E35" s="5" t="inlineStr">
@@ -1716,12 +1716,12 @@
       </c>
       <c r="C36" s="4" t="inlineStr">
         <is>
-          <t>2141r1_cutlet_plot.png</t>
+          <t>2141r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>2141r1_cutlet_data.xlsx</t>
+          <t>2141r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E36" s="5" t="inlineStr">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="C37" s="4" t="inlineStr">
         <is>
-          <t>2142r1_cutlet_plot.png</t>
+          <t>2142r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D37" s="4" t="inlineStr">
         <is>
-          <t>2142r1_cutlet_data.xlsx</t>
+          <t>2142r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E37" s="5" t="inlineStr">
@@ -1790,12 +1790,12 @@
       </c>
       <c r="C38" s="4" t="inlineStr">
         <is>
-          <t>2143r1_cutlet_plot.png</t>
+          <t>2143r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2143r1_cutlet_data.xlsx</t>
+          <t>2143r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E38" s="5" t="inlineStr">
@@ -1827,12 +1827,12 @@
       </c>
       <c r="C39" s="4" t="inlineStr">
         <is>
-          <t>2145r1_cutlet_plot.png</t>
+          <t>2145r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D39" s="4" t="inlineStr">
         <is>
-          <t>2145r1_cutlet_data.xlsx</t>
+          <t>2145r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E39" s="5" t="inlineStr">
@@ -1864,12 +1864,12 @@
       </c>
       <c r="C40" s="4" t="inlineStr">
         <is>
-          <t>2148r1_cutlet_plot.png</t>
+          <t>2148r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>2148r1_cutlet_data.xlsx</t>
+          <t>2148r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E40" s="5" t="inlineStr">
@@ -1901,12 +1901,12 @@
       </c>
       <c r="C41" s="4" t="inlineStr">
         <is>
-          <t>2152r1_cutlet_plot.png</t>
+          <t>2152r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D41" s="4" t="inlineStr">
         <is>
-          <t>2152r1_cutlet_data.xlsx</t>
+          <t>2152r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E41" s="5" t="inlineStr">
@@ -1938,12 +1938,12 @@
       </c>
       <c r="C42" s="4" t="inlineStr">
         <is>
-          <t>2153r1_cutlet_plot.png</t>
+          <t>2153r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>2153r1_cutlet_data.xlsx</t>
+          <t>2153r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E42" s="5" t="inlineStr">
@@ -1975,12 +1975,12 @@
       </c>
       <c r="C43" s="4" t="inlineStr">
         <is>
-          <t>2154r1_cutlet_plot.png</t>
+          <t>2154r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D43" s="4" t="inlineStr">
         <is>
-          <t>2154r1_cutlet_data.xlsx</t>
+          <t>2154r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E43" s="5" t="inlineStr">
@@ -2012,12 +2012,12 @@
       </c>
       <c r="C44" s="4" t="inlineStr">
         <is>
-          <t>2157r1_cutlet_plot.png</t>
+          <t>2157r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2157r1_cutlet_data.xlsx</t>
+          <t>2157r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E44" s="5" t="inlineStr">
@@ -2049,12 +2049,12 @@
       </c>
       <c r="C45" s="4" t="inlineStr">
         <is>
-          <t>2158r2_cutlet_plot.png</t>
+          <t>2158r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D45" s="4" t="inlineStr">
         <is>
-          <t>2158r2_cutlet_data.xlsx</t>
+          <t>2158r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E45" s="5" t="inlineStr">
@@ -2086,12 +2086,12 @@
       </c>
       <c r="C46" s="4" t="inlineStr">
         <is>
-          <t>2160r5_cutlet_plot.png</t>
+          <t>2160r5 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>2160r5_cutlet_data.xlsx</t>
+          <t>2160r5 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E46" s="5" t="inlineStr">
@@ -2123,12 +2123,12 @@
       </c>
       <c r="C47" s="4" t="inlineStr">
         <is>
-          <t>2164r2_cutlet_plot.png</t>
+          <t>2164r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D47" s="4" t="inlineStr">
         <is>
-          <t>2164r2_cutlet_data.xlsx</t>
+          <t>2164r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E47" s="5" t="inlineStr">
@@ -2160,12 +2160,12 @@
       </c>
       <c r="C48" s="4" t="inlineStr">
         <is>
-          <t>2169r2_cutlet_plot.png</t>
+          <t>2169r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>2169r2_cutlet_data.xlsx</t>
+          <t>2169r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E48" s="5" t="inlineStr">
@@ -2197,12 +2197,12 @@
       </c>
       <c r="C49" s="4" t="inlineStr">
         <is>
-          <t>2172r1_cutlet_plot.png</t>
+          <t>2172r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D49" s="4" t="inlineStr">
         <is>
-          <t>2172r1_cutlet_data.xlsx</t>
+          <t>2172r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E49" s="5" t="inlineStr">
@@ -2234,12 +2234,12 @@
       </c>
       <c r="C50" s="4" t="inlineStr">
         <is>
-          <t>2173r1_cutlet_plot.png</t>
+          <t>2173r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>2173r1_cutlet_data.xlsx</t>
+          <t>2173r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E50" s="5" t="inlineStr">
@@ -2271,12 +2271,12 @@
       </c>
       <c r="C51" s="4" t="inlineStr">
         <is>
-          <t>2174r1_cutlet_plot.png</t>
+          <t>2174r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D51" s="4" t="inlineStr">
         <is>
-          <t>2174r1_cutlet_data.xlsx</t>
+          <t>2174r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E51" s="5" t="inlineStr">
@@ -2308,12 +2308,12 @@
       </c>
       <c r="C52" s="4" t="inlineStr">
         <is>
-          <t>2176r06_cutlet_plot.png</t>
+          <t>2176r06 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2176r06_cutlet_data.xlsx</t>
+          <t>2176r06 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E52" s="5" t="inlineStr">
@@ -2345,12 +2345,12 @@
       </c>
       <c r="C53" s="4" t="inlineStr">
         <is>
-          <t>2177r1_cutlet_plot.png</t>
+          <t>2177r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D53" s="4" t="inlineStr">
         <is>
-          <t>2177r1_cutlet_data.xlsx</t>
+          <t>2177r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E53" s="5" t="inlineStr">
@@ -2382,12 +2382,12 @@
       </c>
       <c r="C54" s="4" t="inlineStr">
         <is>
-          <t>2179r1_cutlet_plot.png</t>
+          <t>2179r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>2179r1_cutlet_data.xlsx</t>
+          <t>2179r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E54" s="5" t="inlineStr">
@@ -2419,12 +2419,12 @@
       </c>
       <c r="C55" s="4" t="inlineStr">
         <is>
-          <t>2180r1_cutlet_plot.png</t>
+          <t>2180r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D55" s="4" t="inlineStr">
         <is>
-          <t>2180r1_cutlet_data.xlsx</t>
+          <t>2180r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E55" s="5" t="inlineStr">
@@ -2456,12 +2456,12 @@
       </c>
       <c r="C56" s="4" t="inlineStr">
         <is>
-          <t>2181r1_cutlet_plot.png</t>
+          <t>2181r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2181r1_cutlet_data.xlsx</t>
+          <t>2181r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E56" s="5" t="inlineStr">
@@ -2493,12 +2493,12 @@
       </c>
       <c r="C57" s="4" t="inlineStr">
         <is>
-          <t>2184r1_cutlet_plot.png</t>
+          <t>2184r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D57" s="4" t="inlineStr">
         <is>
-          <t>2184r1_cutlet_data.xlsx</t>
+          <t>2184r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E57" s="5" t="inlineStr">
@@ -2530,12 +2530,12 @@
       </c>
       <c r="C58" s="4" t="inlineStr">
         <is>
-          <t>2185r1_cutlet_plot.png</t>
+          <t>2185r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>2185r1_cutlet_data.xlsx</t>
+          <t>2185r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E58" s="5" t="inlineStr">
@@ -2567,12 +2567,12 @@
       </c>
       <c r="C59" s="4" t="inlineStr">
         <is>
-          <t>2186r1_cutlet_plot.png</t>
+          <t>2186r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D59" s="4" t="inlineStr">
         <is>
-          <t>2186r1_cutlet_data.xlsx</t>
+          <t>2186r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E59" s="5" t="inlineStr">
@@ -2604,12 +2604,12 @@
       </c>
       <c r="C60" s="4" t="inlineStr">
         <is>
-          <t>2188r1_cutlet_plot.png</t>
+          <t>2188r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2188r1_cutlet_data.xlsx</t>
+          <t>2188r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E60" s="5" t="inlineStr">
@@ -2641,12 +2641,12 @@
       </c>
       <c r="C61" s="4" t="inlineStr">
         <is>
-          <t>2190r1_cutlet_plot.png</t>
+          <t>2190r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D61" s="4" t="inlineStr">
         <is>
-          <t>2190r1_cutlet_data.xlsx</t>
+          <t>2190r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E61" s="5" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="C62" s="4" t="inlineStr">
         <is>
-          <t>2192r1_cutlet_plot.png</t>
+          <t>2192r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2192r1_cutlet_data.xlsx</t>
+          <t>2192r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E62" s="5" t="inlineStr">
@@ -2715,12 +2715,12 @@
       </c>
       <c r="C63" s="4" t="inlineStr">
         <is>
-          <t>2193r1_cutlet_plot.png</t>
+          <t>2193r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D63" s="4" t="inlineStr">
         <is>
-          <t>2193r1_cutlet_data.xlsx</t>
+          <t>2193r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E63" s="5" t="inlineStr">
@@ -2752,12 +2752,12 @@
       </c>
       <c r="C64" s="4" t="inlineStr">
         <is>
-          <t>2194r3_cutlet_plot.png</t>
+          <t>2194r3 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>2194r3_cutlet_data.xlsx</t>
+          <t>2194r3 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E64" s="5" t="inlineStr">
@@ -2789,12 +2789,12 @@
       </c>
       <c r="C65" s="4" t="inlineStr">
         <is>
-          <t>2195r1_cutlet_plot.png</t>
+          <t>2195r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D65" s="4" t="inlineStr">
         <is>
-          <t>2195r1_cutlet_data.xlsx</t>
+          <t>2195r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E65" s="5" t="inlineStr">
@@ -2826,12 +2826,12 @@
       </c>
       <c r="C66" s="4" t="inlineStr">
         <is>
-          <t>2196r1_cutlet_plot.png</t>
+          <t>2196r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2196r1_cutlet_data.xlsx</t>
+          <t>2196r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E66" s="5" t="inlineStr">
@@ -2863,12 +2863,12 @@
       </c>
       <c r="C67" s="4" t="inlineStr">
         <is>
-          <t>2198r1_cutlet_plot.png</t>
+          <t>2198r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D67" s="4" t="inlineStr">
         <is>
-          <t>2198r1_cutlet_data.xlsx</t>
+          <t>2198r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E67" s="5" t="inlineStr">
@@ -2900,12 +2900,12 @@
       </c>
       <c r="C68" s="4" t="inlineStr">
         <is>
-          <t>2205r1_cutlet_plot.png</t>
+          <t>2205r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>2205r1_cutlet_data.xlsx</t>
+          <t>2205r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E68" s="5" t="inlineStr">
@@ -2937,12 +2937,12 @@
       </c>
       <c r="C69" s="4" t="inlineStr">
         <is>
-          <t>2206r1_cutlet_plot.png</t>
+          <t>2206r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D69" s="4" t="inlineStr">
         <is>
-          <t>2206r1_cutlet_data.xlsx</t>
+          <t>2206r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E69" s="5" t="inlineStr">
@@ -2974,12 +2974,12 @@
       </c>
       <c r="C70" s="4" t="inlineStr">
         <is>
-          <t>2207r2_cutlet_plot.png</t>
+          <t>2207r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2207r2_cutlet_data.xlsx</t>
+          <t>2207r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E70" s="5" t="inlineStr">
@@ -3011,12 +3011,12 @@
       </c>
       <c r="C71" s="4" t="inlineStr">
         <is>
-          <t>2208r1_cutlet_plot.png</t>
+          <t>2208r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D71" s="4" t="inlineStr">
         <is>
-          <t>2208r1_cutlet_data.xlsx</t>
+          <t>2208r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E71" s="5" t="inlineStr">
@@ -3048,12 +3048,12 @@
       </c>
       <c r="C72" s="4" t="inlineStr">
         <is>
-          <t>2209r1_cutlet_plot.png</t>
+          <t>2209r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2209r1_cutlet_data.xlsx</t>
+          <t>2209r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E72" s="5" t="inlineStr">
@@ -3085,12 +3085,12 @@
       </c>
       <c r="C73" s="4" t="inlineStr">
         <is>
-          <t>2210r1_cutlet_plot.png</t>
+          <t>2210r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D73" s="4" t="inlineStr">
         <is>
-          <t>2210r1_cutlet_data.xlsx</t>
+          <t>2210r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E73" s="5" t="inlineStr">
@@ -3122,12 +3122,12 @@
       </c>
       <c r="C74" s="4" t="inlineStr">
         <is>
-          <t>2216r1_cutlet_plot.png</t>
+          <t>2216r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>2216r1_cutlet_data.xlsx</t>
+          <t>2216r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E74" s="5" t="inlineStr">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="C75" s="4" t="inlineStr">
         <is>
-          <t>2217r1_cutlet_plot.png</t>
+          <t>2217r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D75" s="4" t="inlineStr">
         <is>
-          <t>2217r1_cutlet_data.xlsx</t>
+          <t>2217r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E75" s="5" t="inlineStr">
@@ -3196,12 +3196,12 @@
       </c>
       <c r="C76" s="4" t="inlineStr">
         <is>
-          <t>2218r1_cutlet_plot.png</t>
+          <t>2218r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>2218r1_cutlet_data.xlsx</t>
+          <t>2218r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E76" s="5" t="inlineStr">
@@ -3233,12 +3233,12 @@
       </c>
       <c r="C77" s="4" t="inlineStr">
         <is>
-          <t>2220r1_cutlet_plot.png</t>
+          <t>2220r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D77" s="4" t="inlineStr">
         <is>
-          <t>2220r1_cutlet_data.xlsx</t>
+          <t>2220r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E77" s="5" t="inlineStr">
@@ -3270,12 +3270,12 @@
       </c>
       <c r="C78" s="4" t="inlineStr">
         <is>
-          <t>2224r1_cutlet_plot.png</t>
+          <t>2224r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>2224r1_cutlet_data.xlsx</t>
+          <t>2224r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E78" s="5" t="inlineStr">
@@ -3307,12 +3307,12 @@
       </c>
       <c r="C79" s="4" t="inlineStr">
         <is>
-          <t>2225r1_cutlet_plot.png</t>
+          <t>2225r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D79" s="4" t="inlineStr">
         <is>
-          <t>2225r1_cutlet_data.xlsx</t>
+          <t>2225r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E79" s="5" t="inlineStr">
@@ -3344,12 +3344,12 @@
       </c>
       <c r="C80" s="4" t="inlineStr">
         <is>
-          <t>2226r1_cutlet_plot.png</t>
+          <t>2226r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>2226r1_cutlet_data.xlsx</t>
+          <t>2226r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E80" s="5" t="inlineStr">
@@ -3381,12 +3381,12 @@
       </c>
       <c r="C81" s="4" t="inlineStr">
         <is>
-          <t>2227r1_cutlet_plot.png</t>
+          <t>2227r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D81" s="4" t="inlineStr">
         <is>
-          <t>2227r1_cutlet_data.xlsx</t>
+          <t>2227r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E81" s="5" t="inlineStr">
@@ -3418,12 +3418,12 @@
       </c>
       <c r="C82" s="4" t="inlineStr">
         <is>
-          <t>2231r1_cutlet_plot.png</t>
+          <t>2231r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2231r1_cutlet_data.xlsx</t>
+          <t>2231r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E82" s="5" t="inlineStr">
@@ -3455,12 +3455,12 @@
       </c>
       <c r="C83" s="4" t="inlineStr">
         <is>
-          <t>2232r1_cutlet_plot.png</t>
+          <t>2232r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D83" s="4" t="inlineStr">
         <is>
-          <t>2232r1_cutlet_data.xlsx</t>
+          <t>2232r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E83" s="5" t="inlineStr">
@@ -3492,12 +3492,12 @@
       </c>
       <c r="C84" s="4" t="inlineStr">
         <is>
-          <t>2234r1_cutlet_plot.png</t>
+          <t>2234r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>2234r1_cutlet_data.xlsx</t>
+          <t>2234r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E84" s="5" t="inlineStr">
@@ -3529,12 +3529,12 @@
       </c>
       <c r="C85" s="4" t="inlineStr">
         <is>
-          <t>2235r1_cutlet_plot.png</t>
+          <t>2235r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D85" s="4" t="inlineStr">
         <is>
-          <t>2235r1_cutlet_data.xlsx</t>
+          <t>2235r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E85" s="5" t="inlineStr">
@@ -3566,12 +3566,12 @@
       </c>
       <c r="C86" s="4" t="inlineStr">
         <is>
-          <t>2236r1_cutlet_plot.png</t>
+          <t>2236r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>2236r1_cutlet_data.xlsx</t>
+          <t>2236r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E86" s="5" t="inlineStr">
@@ -3603,12 +3603,12 @@
       </c>
       <c r="C87" s="4" t="inlineStr">
         <is>
-          <t>2240r1_cutlet_plot.png</t>
+          <t>2240r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D87" s="4" t="inlineStr">
         <is>
-          <t>2240r1_cutlet_data.xlsx</t>
+          <t>2240r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E87" s="5" t="inlineStr">
@@ -3640,12 +3640,12 @@
       </c>
       <c r="C88" s="4" t="inlineStr">
         <is>
-          <t>2241r1_cutlet_plot.png</t>
+          <t>2241r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2241r1_cutlet_data.xlsx</t>
+          <t>2241r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E88" s="5" t="inlineStr">
@@ -3677,12 +3677,12 @@
       </c>
       <c r="C89" s="4" t="inlineStr">
         <is>
-          <t>2242r0_cutlet_plot.png</t>
+          <t>2242r0 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D89" s="4" t="inlineStr">
         <is>
-          <t>2242r0_cutlet_data.xlsx</t>
+          <t>2242r0 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E89" s="5" t="inlineStr">
@@ -3714,12 +3714,12 @@
       </c>
       <c r="C90" s="4" t="inlineStr">
         <is>
-          <t>2247r1_cutlet_plot.png</t>
+          <t>2247r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2247r1_cutlet_data.xlsx</t>
+          <t>2247r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E90" s="5" t="inlineStr">
@@ -3751,12 +3751,12 @@
       </c>
       <c r="C91" s="4" t="inlineStr">
         <is>
-          <t>2249r1_cutlet_plot.png</t>
+          <t>2249r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D91" s="4" t="inlineStr">
         <is>
-          <t>2249r1_cutlet_data.xlsx</t>
+          <t>2249r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E91" s="5" t="inlineStr">
@@ -3788,12 +3788,12 @@
       </c>
       <c r="C92" s="4" t="inlineStr">
         <is>
-          <t>2251r1_cutlet_plot.png</t>
+          <t>2251r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2251r1_cutlet_data.xlsx</t>
+          <t>2251r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E92" s="5" t="inlineStr">
@@ -3825,12 +3825,12 @@
       </c>
       <c r="C93" s="4" t="inlineStr">
         <is>
-          <t>2252r1_cutlet_plot.png</t>
+          <t>2252r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D93" s="4" t="inlineStr">
         <is>
-          <t>2252r1_cutlet_data.xlsx</t>
+          <t>2252r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E93" s="5" t="inlineStr">
@@ -3862,12 +3862,12 @@
       </c>
       <c r="C94" s="4" t="inlineStr">
         <is>
-          <t>2256r2_cutlet_plot.png</t>
+          <t>2256r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>2256r2_cutlet_data.xlsx</t>
+          <t>2256r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E94" s="5" t="inlineStr">
@@ -3899,12 +3899,12 @@
       </c>
       <c r="C95" s="4" t="inlineStr">
         <is>
-          <t>2265r0 w Rippers_cutlet_plot.png</t>
+          <t>2265r0 w Rippers @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D95" s="4" t="inlineStr">
         <is>
-          <t>2265r0 w Rippers_cutlet_data.xlsx</t>
+          <t>2265r0 w Rippers @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E95" s="5" t="inlineStr">
@@ -3936,12 +3936,12 @@
       </c>
       <c r="C96" s="4" t="inlineStr">
         <is>
-          <t>2265r1_cutlet_plot.png</t>
+          <t>2265r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>2265r1_cutlet_data.xlsx</t>
+          <t>2265r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E96" s="5" t="inlineStr">
@@ -3973,12 +3973,12 @@
       </c>
       <c r="C97" s="4" t="inlineStr">
         <is>
-          <t>2266r1_cutlet_plot.png</t>
+          <t>2266r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D97" s="4" t="inlineStr">
         <is>
-          <t>2266r1_cutlet_data.xlsx</t>
+          <t>2266r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E97" s="5" t="inlineStr">
@@ -4010,12 +4010,12 @@
       </c>
       <c r="C98" s="4" t="inlineStr">
         <is>
-          <t>2267r1_cutlet_plot.png</t>
+          <t>2267r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D98" s="4" t="inlineStr">
         <is>
-          <t>2267r1_cutlet_data.xlsx</t>
+          <t>2267r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E98" s="5" t="inlineStr">
@@ -4047,12 +4047,12 @@
       </c>
       <c r="C99" s="4" t="inlineStr">
         <is>
-          <t>2268r2_cutlet_plot.png</t>
+          <t>2268r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D99" s="4" t="inlineStr">
         <is>
-          <t>2268r2_cutlet_data.xlsx</t>
+          <t>2268r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E99" s="5" t="inlineStr">
@@ -4084,12 +4084,12 @@
       </c>
       <c r="C100" s="4" t="inlineStr">
         <is>
-          <t>2268r3_cutlet_plot.png</t>
+          <t>2268r3 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>2268r3_cutlet_data.xlsx</t>
+          <t>2268r3 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E100" s="5" t="inlineStr">
@@ -4121,12 +4121,12 @@
       </c>
       <c r="C101" s="4" t="inlineStr">
         <is>
-          <t>2270r1_cutlet_plot.png</t>
+          <t>2270r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D101" s="4" t="inlineStr">
         <is>
-          <t>2270r1_cutlet_data.xlsx</t>
+          <t>2270r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E101" s="5" t="inlineStr">
@@ -4158,12 +4158,12 @@
       </c>
       <c r="C102" s="4" t="inlineStr">
         <is>
-          <t>2272r2_cutlet_plot.png</t>
+          <t>2272r2 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D102" s="4" t="inlineStr">
         <is>
-          <t>2272r2_cutlet_data.xlsx</t>
+          <t>2272r2 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E102" s="5" t="inlineStr">
@@ -4195,12 +4195,12 @@
       </c>
       <c r="C103" s="4" t="inlineStr">
         <is>
-          <t>2362r00_cutlet_plot.png</t>
+          <t>2362r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D103" s="4" t="inlineStr">
         <is>
-          <t>2362r00_cutlet_data.xlsx</t>
+          <t>2362r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E103" s="5" t="inlineStr">
@@ -4232,12 +4232,12 @@
       </c>
       <c r="C104" s="4" t="inlineStr">
         <is>
-          <t>2381r01_cutlet_plot.png</t>
+          <t>2381r01 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D104" s="4" t="inlineStr">
         <is>
-          <t>2381r01_cutlet_data.xlsx</t>
+          <t>2381r01 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E104" s="5" t="inlineStr">
@@ -4269,12 +4269,12 @@
       </c>
       <c r="C105" s="4" t="inlineStr">
         <is>
-          <t>2381r1_cutlet_plot.png</t>
+          <t>2381r1 @ 1.360 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D105" s="4" t="inlineStr">
         <is>
-          <t>2381r1_cutlet_data.xlsx</t>
+          <t>2381r1 @ 1.360 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E105" s="5" t="inlineStr">
@@ -4306,12 +4306,12 @@
       </c>
       <c r="C106" s="4" t="inlineStr">
         <is>
-          <t>2556r00_cutlet_plot.png</t>
+          <t>2556r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D106" s="4" t="inlineStr">
         <is>
-          <t>2556r00_cutlet_data.xlsx</t>
+          <t>2556r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E106" s="5" t="inlineStr">
@@ -4343,12 +4343,12 @@
       </c>
       <c r="C107" s="4" t="inlineStr">
         <is>
-          <t>2556r00 XH23F_cutlet_plot.png</t>
+          <t>2556r00 XH23F @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D107" s="4" t="inlineStr">
         <is>
-          <t>2556r00 XH23F_cutlet_data.xlsx</t>
+          <t>2556r00 XH23F @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E107" s="5" t="inlineStr">
@@ -4380,12 +4380,12 @@
       </c>
       <c r="C108" s="4" t="inlineStr">
         <is>
-          <t>2746r00_cutlet_plot.png</t>
+          <t>2746r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D108" s="4" t="inlineStr">
         <is>
-          <t>2746r00_cutlet_data.xlsx</t>
+          <t>2746r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E108" s="5" t="inlineStr">
@@ -4417,12 +4417,12 @@
       </c>
       <c r="C109" s="4" t="inlineStr">
         <is>
-          <t>3219r00_cutlet_plot.png</t>
+          <t>3219r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D109" s="4" t="inlineStr">
         <is>
-          <t>3219r00_cutlet_data.xlsx</t>
+          <t>3219r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E109" s="5" t="inlineStr">
@@ -4454,12 +4454,12 @@
       </c>
       <c r="C110" s="4" t="inlineStr">
         <is>
-          <t>3336r00_cutlet_plot.png</t>
+          <t>3336r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D110" s="4" t="inlineStr">
         <is>
-          <t>3336r00_cutlet_data.xlsx</t>
+          <t>3336r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E110" s="5" t="inlineStr">
@@ -4491,12 +4491,12 @@
       </c>
       <c r="C111" s="4" t="inlineStr">
         <is>
-          <t>3336r00c3_cutlet_plot.png</t>
+          <t>3336r00c3 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D111" s="4" t="inlineStr">
         <is>
-          <t>3336r00c3_cutlet_data.xlsx</t>
+          <t>3336r00c3 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E111" s="5" t="inlineStr">
@@ -4528,12 +4528,12 @@
       </c>
       <c r="C112" s="4" t="inlineStr">
         <is>
-          <t>3449r00_cutlet_plot.png</t>
+          <t>3449r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D112" s="4" t="inlineStr">
         <is>
-          <t>3449r00_cutlet_data.xlsx</t>
+          <t>3449r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E112" s="5" t="inlineStr">
@@ -4565,12 +4565,12 @@
       </c>
       <c r="C113" s="4" t="inlineStr">
         <is>
-          <t>3943r1_cutlet_plot.png</t>
+          <t>3943r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D113" s="4" t="inlineStr">
         <is>
-          <t>3943r1_cutlet_data.xlsx</t>
+          <t>3943r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E113" s="5" t="inlineStr">
@@ -4602,12 +4602,12 @@
       </c>
       <c r="C114" s="4" t="inlineStr">
         <is>
-          <t>4149r00_cutlet_plot.png</t>
+          <t>4149r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D114" s="4" t="inlineStr">
         <is>
-          <t>4149r00_cutlet_data.xlsx</t>
+          <t>4149r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E114" s="5" t="inlineStr">
@@ -4639,12 +4639,12 @@
       </c>
       <c r="C115" s="4" t="inlineStr">
         <is>
-          <t>4206r1_cutlet_plot.png</t>
+          <t>4206r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D115" s="4" t="inlineStr">
         <is>
-          <t>4206r1_cutlet_data.xlsx</t>
+          <t>4206r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E115" s="5" t="inlineStr">
@@ -4676,12 +4676,12 @@
       </c>
       <c r="C116" s="4" t="inlineStr">
         <is>
-          <t>4288r00_cutlet_plot.png</t>
+          <t>4288r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D116" s="4" t="inlineStr">
         <is>
-          <t>4288r00_cutlet_data.xlsx</t>
+          <t>4288r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E116" s="5" t="inlineStr">
@@ -4713,12 +4713,12 @@
       </c>
       <c r="C117" s="4" t="inlineStr">
         <is>
-          <t>4538r0_cutlet_plot.png</t>
+          <t>4538r0 @ 0.333 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D117" s="4" t="inlineStr">
         <is>
-          <t>4538r0_cutlet_data.xlsx</t>
+          <t>4538r0 @ 0.333 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E117" s="5" t="inlineStr">
@@ -4750,12 +4750,12 @@
       </c>
       <c r="C118" s="4" t="inlineStr">
         <is>
-          <t>4538r00_cutlet_plot.png</t>
+          <t>4538r00 @ 0.153 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D118" s="4" t="inlineStr">
         <is>
-          <t>4538r00_cutlet_data.xlsx</t>
+          <t>4538r00 @ 0.153 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E118" s="5" t="inlineStr">
@@ -4787,12 +4787,12 @@
       </c>
       <c r="C119" s="4" t="inlineStr">
         <is>
-          <t>4720r01_cutlet_plot.png</t>
+          <t>4720r01 @ 0.300 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D119" s="4" t="inlineStr">
         <is>
-          <t>4720r01_cutlet_data.xlsx</t>
+          <t>4720r01 @ 0.300 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E119" s="5" t="inlineStr">
@@ -4824,12 +4824,12 @@
       </c>
       <c r="C120" s="4" t="inlineStr">
         <is>
-          <t>4720r1_cutlet_plot.png</t>
+          <t>4720r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D120" s="4" t="inlineStr">
         <is>
-          <t>4720r1_cutlet_data.xlsx</t>
+          <t>4720r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E120" s="5" t="inlineStr">
@@ -4861,12 +4861,12 @@
       </c>
       <c r="C121" s="4" t="inlineStr">
         <is>
-          <t>4796r00_cutlet_plot.png</t>
+          <t>4796r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D121" s="4" t="inlineStr">
         <is>
-          <t>4796r00_cutlet_data.xlsx</t>
+          <t>4796r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E121" s="5" t="inlineStr">
@@ -4898,12 +4898,12 @@
       </c>
       <c r="C122" s="4" t="inlineStr">
         <is>
-          <t>5131r00_cutlet_plot.png</t>
+          <t>5131r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D122" s="4" t="inlineStr">
         <is>
-          <t>5131r00_cutlet_data.xlsx</t>
+          <t>5131r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E122" s="5" t="inlineStr">
@@ -4935,12 +4935,12 @@
       </c>
       <c r="C123" s="4" t="inlineStr">
         <is>
-          <t>5132r00_cutlet_plot.png</t>
+          <t>5132r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D123" s="4" t="inlineStr">
         <is>
-          <t>5132r00_cutlet_data.xlsx</t>
+          <t>5132r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E123" s="5" t="inlineStr">
@@ -4972,12 +4972,12 @@
       </c>
       <c r="C124" s="4" t="inlineStr">
         <is>
-          <t>5481r0 Rev_cutlet_plot.png</t>
+          <t>5481r0 Rev @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D124" s="4" t="inlineStr">
         <is>
-          <t>5481r0 Rev_cutlet_data.xlsx</t>
+          <t>5481r0 Rev @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E124" s="5" t="inlineStr">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C125" s="4" t="inlineStr">
         <is>
-          <t>5646r00_cutlet_plot.png</t>
+          <t>5646r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D125" s="4" t="inlineStr">
         <is>
-          <t>5646r00_cutlet_data.xlsx</t>
+          <t>5646r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E125" s="5" t="inlineStr">
@@ -5046,12 +5046,12 @@
       </c>
       <c r="C126" s="4" t="inlineStr">
         <is>
-          <t>5674r00_cutlet_plot.png</t>
+          <t>5674r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D126" s="4" t="inlineStr">
         <is>
-          <t>5674r00_cutlet_data.xlsx</t>
+          <t>5674r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E126" s="5" t="inlineStr">
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C127" s="4" t="inlineStr">
         <is>
-          <t>5749r00_cutlet_plot.png</t>
+          <t>5749r00 @ 0.167 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D127" s="4" t="inlineStr">
         <is>
-          <t>5749r00_cutlet_data.xlsx</t>
+          <t>5749r00 @ 0.167 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E127" s="5" t="inlineStr">
@@ -5120,12 +5120,12 @@
       </c>
       <c r="C128" s="4" t="inlineStr">
         <is>
-          <t>5911r00_cutlet_plot.png</t>
+          <t>5911r00 @ 0.190 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D128" s="4" t="inlineStr">
         <is>
-          <t>5911r00_cutlet_data.xlsx</t>
+          <t>5911r00 @ 0.190 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E128" s="5" t="inlineStr">
@@ -5157,12 +5157,12 @@
       </c>
       <c r="C129" s="4" t="inlineStr">
         <is>
-          <t>6135r00_cutlet_plot.png</t>
+          <t>6135r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D129" s="4" t="inlineStr">
         <is>
-          <t>6135r00_cutlet_data.xlsx</t>
+          <t>6135r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E129" s="5" t="inlineStr">
@@ -5194,12 +5194,12 @@
       </c>
       <c r="C130" s="4" t="inlineStr">
         <is>
-          <t>6150r00_cutlet_plot.png</t>
+          <t>6150r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D130" s="4" t="inlineStr">
         <is>
-          <t>6150r00_cutlet_data.xlsx</t>
+          <t>6150r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E130" s="5" t="inlineStr">
@@ -5231,12 +5231,12 @@
       </c>
       <c r="C131" s="4" t="inlineStr">
         <is>
-          <t>6150r01_cutlet_plot.png</t>
+          <t>6150r01 @ 0.840 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D131" s="4" t="inlineStr">
         <is>
-          <t>6150r01_cutlet_data.xlsx</t>
+          <t>6150r01 @ 0.840 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E131" s="5" t="inlineStr">
@@ -5268,12 +5268,12 @@
       </c>
       <c r="C132" s="4" t="inlineStr">
         <is>
-          <t>6207r1_cutlet_plot.png</t>
+          <t>6207r1 @ 1.360 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D132" s="4" t="inlineStr">
         <is>
-          <t>6207r1_cutlet_data.xlsx</t>
+          <t>6207r1 @ 1.360 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E132" s="5" t="inlineStr">
@@ -5305,12 +5305,12 @@
       </c>
       <c r="C133" s="4" t="inlineStr">
         <is>
-          <t>6513r0_cutlet_plot.png</t>
+          <t>6513r0 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D133" s="4" t="inlineStr">
         <is>
-          <t>6513r0_cutlet_data.xlsx</t>
+          <t>6513r0 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E133" s="5" t="inlineStr">
@@ -5342,12 +5342,12 @@
       </c>
       <c r="C134" s="4" t="inlineStr">
         <is>
-          <t>6513r00_cutlet_plot.png</t>
+          <t>6513r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D134" s="4" t="inlineStr">
         <is>
-          <t>6513r00_cutlet_data.xlsx</t>
+          <t>6513r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E134" s="5" t="inlineStr">
@@ -5379,12 +5379,12 @@
       </c>
       <c r="C135" s="4" t="inlineStr">
         <is>
-          <t>6653r00_cutlet_plot.png</t>
+          <t>6653r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D135" s="4" t="inlineStr">
         <is>
-          <t>6653r00_cutlet_data.xlsx</t>
+          <t>6653r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E135" s="5" t="inlineStr">
@@ -5416,12 +5416,12 @@
       </c>
       <c r="C136" s="4" t="inlineStr">
         <is>
-          <t>6841r00_cutlet_plot.png</t>
+          <t>6841r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D136" s="4" t="inlineStr">
         <is>
-          <t>6841r00_cutlet_data.xlsx</t>
+          <t>6841r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E136" s="5" t="inlineStr">
@@ -5453,12 +5453,12 @@
       </c>
       <c r="C137" s="4" t="inlineStr">
         <is>
-          <t>7182r00_cutlet_plot.png</t>
+          <t>7182r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D137" s="4" t="inlineStr">
         <is>
-          <t>7182r00_cutlet_data.xlsx</t>
+          <t>7182r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E137" s="5" t="inlineStr">
@@ -5490,12 +5490,12 @@
       </c>
       <c r="C138" s="4" t="inlineStr">
         <is>
-          <t>7273r00_cutlet_plot.png</t>
+          <t>7273r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D138" s="4" t="inlineStr">
         <is>
-          <t>7273r00_cutlet_data.xlsx</t>
+          <t>7273r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E138" s="5" t="inlineStr">
@@ -5527,12 +5527,12 @@
       </c>
       <c r="C139" s="4" t="inlineStr">
         <is>
-          <t>7823r00_cutlet_plot.png</t>
+          <t>7823r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D139" s="4" t="inlineStr">
         <is>
-          <t>7823r00_cutlet_data.xlsx</t>
+          <t>7823r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E139" s="5" t="inlineStr">
@@ -5564,12 +5564,12 @@
       </c>
       <c r="C140" s="4" t="inlineStr">
         <is>
-          <t>8479r1_cutlet_plot.png</t>
+          <t>8479r1 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D140" s="4" t="inlineStr">
         <is>
-          <t>8479r1_cutlet_data.xlsx</t>
+          <t>8479r1 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E140" s="5" t="inlineStr">
@@ -5601,12 +5601,12 @@
       </c>
       <c r="C141" s="4" t="inlineStr">
         <is>
-          <t>8896r00_cutlet_plot.png</t>
+          <t>8896r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D141" s="4" t="inlineStr">
         <is>
-          <t>8896r00_cutlet_data.xlsx</t>
+          <t>8896r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E141" s="5" t="inlineStr">
@@ -5638,12 +5638,12 @@
       </c>
       <c r="C142" s="4" t="inlineStr">
         <is>
-          <t>9023r00_cutlet_plot.png</t>
+          <t>9023r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D142" s="4" t="inlineStr">
         <is>
-          <t>9023r00_cutlet_data.xlsx</t>
+          <t>9023r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E142" s="5" t="inlineStr">
@@ -5675,12 +5675,12 @@
       </c>
       <c r="C143" s="4" t="inlineStr">
         <is>
-          <t>9387r00_cutlet_plot.png</t>
+          <t>9387r00 @ 0.208 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D143" s="4" t="inlineStr">
         <is>
-          <t>9387r00_cutlet_data.xlsx</t>
+          <t>9387r00 @ 0.208 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E143" s="5" t="inlineStr">
@@ -5712,12 +5712,12 @@
       </c>
       <c r="C144" s="4" t="inlineStr">
         <is>
-          <t>9692r00_cutlet_plot.png</t>
+          <t>9692r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D144" s="4" t="inlineStr">
         <is>
-          <t>9692r00_cutlet_data.xlsx</t>
+          <t>9692r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E144" s="5" t="inlineStr">
@@ -5749,12 +5749,12 @@
       </c>
       <c r="C145" s="4" t="inlineStr">
         <is>
-          <t>9944r00_cutlet_plot.png</t>
+          <t>9944r00 @ 0.250 IPR_cutlet_plot.png</t>
         </is>
       </c>
       <c r="D145" s="4" t="inlineStr">
         <is>
-          <t>9944r00_cutlet_data.xlsx</t>
+          <t>9944r00 @ 0.250 IPR_cutlet_data.xlsx</t>
         </is>
       </c>
       <c r="E145" s="5" t="inlineStr">

</xml_diff>